<commit_message>
Improve plot tick generation and number parsing
Add nicer tick computation and axis range handling: introduce niceStep and niceTickValues to produce human-friendly tick intervals, extend buildTicks to accept optional forceMin/forceMax and return tick ranges, and update baseLayout to use these for enforcing zero starts and y_max behavior instead of ad-hoc range logic. Also improve parseEditableCell to normalize European decimal commas (e.g. "2,4" → "2.4") before numeric parsing. Minor project updates: add CLAUDE.md to .gitignore and a binary update to Hoppler/Hoppler.xlsx.
</commit_message>
<xml_diff>
--- a/Hoppler/Hoppler.xlsx
+++ b/Hoppler/Hoppler.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t xml:space="preserve">temp</t>
   </si>
@@ -38,20 +38,25 @@
   </si>
   <si>
     <t xml:space="preserve">delta eta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eta (Pas)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -111,13 +116,25 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -243,134 +260,166 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.32"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="H1" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>26.79</v>
       </c>
-      <c r="C2" s="1" t="n">
+      <c r="C2" s="2" t="n">
         <v>0.1318</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="3" t="n">
         <f aca="false">$C$2*B2*(8130-1260/(1+A2*0.0005))/1000</f>
         <v>24.3036628367442</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="3" t="n">
         <f aca="false">$C$2*B2*(8130-1260)/1000</f>
         <v>24.25743414</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="F2" s="4"/>
+      <c r="G2" s="3" t="n">
         <f aca="false">-$C$2*(1260*0.0005/(1+0.0005*A2)^2)*0.1+$C$2*(8130-1260/(1+0.0005*A2))/1000</f>
         <v>0.89905985825086</v>
       </c>
+      <c r="H2" s="4" t="n">
+        <f aca="false">D2/1000</f>
+        <v>0.0243036628367442</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>32.6</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>12.04</v>
       </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="0" t="n">
+      <c r="C3" s="2"/>
+      <c r="D3" s="3" t="n">
         <f aca="false">$C$2*B3*(8130-1260/(1+A3*0.0005))/1000</f>
         <v>10.9338791012181</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="3" t="n">
         <f aca="false">$C$2*B3*(8130-1260)/1000</f>
         <v>10.90181064</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="F3" s="4"/>
+      <c r="G3" s="3" t="n">
         <f aca="false">-$C$2*(1260*0.0005/(1+0.0005*A3)^2)*0.1+$C$2*(8130-1260/(1+0.0005*A3))/1000</f>
         <v>0.900090306870838</v>
       </c>
+      <c r="H3" s="4" t="n">
+        <f aca="false">D3/1000</f>
+        <v>0.0109338791012181</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>6.06</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="0" t="n">
+      <c r="C4" s="2"/>
+      <c r="D4" s="3" t="n">
         <f aca="false">$C$2*B4*(8130-1260/(1+A4*0.0005))/1000</f>
         <v>5.5083055554185</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="3" t="n">
         <f aca="false">$C$2*B4*(8130-1260)/1000</f>
         <v>5.48712396</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="F4" s="4"/>
+      <c r="G4" s="3" t="n">
         <f aca="false">-$C$2*(1260*0.0005/(1+0.0005*A4)^2)*0.1+$C$2*(8130-1260/(1+0.0005*A4))/1000</f>
         <v>0.901003765676717</v>
       </c>
+      <c r="H4" s="4" t="n">
+        <f aca="false">D4/1000</f>
+        <v>0.0055083055554185</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>52.5</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>3.73</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="0" t="n">
+      <c r="C5" s="2"/>
+      <c r="D5" s="3" t="n">
         <f aca="false">$C$2*B5*(8130-1260/(1+A5*0.0005))/1000</f>
         <v>3.39323240221681</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="3" t="n">
         <f aca="false">$C$2*B5*(8130-1260)/1000</f>
         <v>3.37738818</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="F5" s="4"/>
+      <c r="G5" s="3" t="n">
         <f aca="false">-$C$2*(1260*0.0005/(1+0.0005*A5)^2)*0.1+$C$2*(8130-1260/(1+0.0005*A5))/1000</f>
         <v>0.901829726224369</v>
       </c>
+      <c r="H5" s="4" t="n">
+        <f aca="false">D5/1000</f>
+        <v>0.00339323240221681</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>62</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>2.63</v>
       </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="0" t="n">
+      <c r="C6" s="2"/>
+      <c r="D6" s="3" t="n">
         <f aca="false">$C$2*B6*(8130-1260/(1+A6*0.0005))/1000</f>
         <v>2.39450799904947</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="3" t="n">
         <f aca="false">$C$2*B6*(8130-1260)/1000</f>
         <v>2.38137558</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="F6" s="4"/>
+      <c r="G6" s="3" t="n">
         <f aca="false">-$C$2*(1260*0.0005/(1+0.0005*A6)^2)*0.1+$C$2*(8130-1260/(1+0.0005*A6))/1000</f>
         <v>0.902647739826767</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <f aca="false">D6/1000</f>
+        <v>0.00239450799904947</v>
       </c>
     </row>
   </sheetData>

</xml_diff>